<commit_message>
sprint 9 + 10 - MVP
</commit_message>
<xml_diff>
--- a/docs/samples/teaching-assignments-import-sample.xlsx
+++ b/docs/samples/teaching-assignments-import-sample.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>email_gv</t>
   </si>
@@ -23,33 +23,39 @@
     <t>ngay_phan_cong</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>TOAN-10A1</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>VAN-10A1</t>
+  </si>
+  <si>
     <t>nguyenthilan.import@demo.edu.vn</t>
   </si>
   <si>
-    <t>TOAN-10A1</t>
-  </si>
-  <si>
-    <t>2025-09-01</t>
+    <t>TOAN-11A1</t>
   </si>
   <si>
     <t>tranvanhung.import@demo.edu.vn</t>
   </si>
   <si>
-    <t>VAN-10A1</t>
+    <t>VAN-11A1</t>
   </si>
   <si>
     <t>lethimai.import@demo.edu.vn</t>
   </si>
   <si>
-    <t>ANH-10A1</t>
+    <t>TOAN-12A1</t>
   </si>
   <si>
     <t>Hướng dẫn import phân công giảng dạy</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Cột bắt buộc: email_gv, ma_lop_mon, ngay_phan_cong (YYYY-MM-DD)</t>
   </si>
   <si>
@@ -72,6 +78,18 @@
   </si>
   <si>
     <t>- Nếu phân công đã tồn tại nhưng INACTIVE sẽ được kích hoạt lại</t>
+  </si>
+  <si>
+    <t>Tải mẫu kèm học kỳ:</t>
+  </si>
+  <si>
+    <t>- Khối đầu cấp (vd. 10): email_gv để trống — điền GV mới</t>
+  </si>
+  <si>
+    <t>- Khối 11/12: email_gv lấy từ phân công ACTIVE HK2 năm trước (cùng mã lớp HC + mã môn)</t>
+  </si>
+  <si>
+    <t>File mẫu tham khảo: docs/samples/teaching-assignments-import-sample.xlsx</t>
   </si>
 </sst>
 </file>
@@ -110,10 +128,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,14 +478,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,36 +496,58 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -513,7 +559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
@@ -521,57 +567,97 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>